<commit_message>
local food db setting up
</commit_message>
<xml_diff>
--- a/backend/data/food/raw/arugam_bay/arugam_bay_local_food_recommendation_dataset/arugam_bay_local_food_dataset.xlsx
+++ b/backend/data/food/raw/arugam_bay/arugam_bay_local_food_recommendation_dataset/arugam_bay_local_food_dataset.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_items" sheetId="1" r:id="R35dac9da3e5f4552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_places" sheetId="2" r:id="R0ce704e1f1684d24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_place_dishes" sheetId="3" r:id="R0833c94e2b3c4e85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="social_recommendations" sheetId="4" r:id="R7b4b18eda4a9406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="city_food_profile" sheetId="5" r:id="Rd19a6b72c1214c00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recommendation_tags" sheetId="6" r:id="Ra519d264185544fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_registry" sheetId="7" r:id="R257f8151a4b94cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="evaluation_queries" sheetId="8" r:id="R15a04441b2b74d57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_items" sheetId="1" r:id="Ra86acf73ddd6454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_places" sheetId="2" r:id="R557dc5cc540f4032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="food_place_dishes" sheetId="3" r:id="Rfd6c9ea87dcb4261"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="social_recommendations" sheetId="4" r:id="R253734a55e1d47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="city_food_profile" sheetId="5" r:id="R7a3525ae06a54257"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recommendation_tags" sheetId="6" r:id="Rf0c869c116e8491f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="source_registry" sheetId="7" r:id="R861030d0b1d94dc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="evaluation_queries" sheetId="8" r:id="R12422b91b7274395"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -29,6 +29,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -52,7 +57,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -82,6 +87,17 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1545,25 +1561,26 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="30" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="16" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="16" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="16" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="7.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="9.5" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="13.75" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="5" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="11" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="28" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="28" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="28" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="28" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="28" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="10.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="8.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1574,54 +1591,57 @@
         <x:v>place_name</x:v>
       </x:c>
       <x:c r="C1" s="10" t="str">
-        <x:v>arugam_bay_area</x:v>
+        <x:v>city</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
+        <x:v>area</x:v>
+      </x:c>
+      <x:c r="E1" s="10" t="str">
         <x:v>address</x:v>
       </x:c>
-      <x:c r="E1" s="10" t="str">
+      <x:c r="F1" s="10" t="str">
         <x:v>place_type</x:v>
       </x:c>
-      <x:c r="F1" s="10" t="str">
+      <x:c r="G1" s="10" t="str">
         <x:v>cuisine_focus</x:v>
       </x:c>
-      <x:c r="G1" s="10" t="str">
+      <x:c r="H1" s="10" t="str">
         <x:v>local_food_strength</x:v>
       </x:c>
-      <x:c r="H1" s="10" t="str">
+      <x:c r="I1" s="10" t="str">
         <x:v>dietary_strength</x:v>
       </x:c>
-      <x:c r="I1" s="10" t="str">
+      <x:c r="J1" s="10" t="str">
         <x:v>price_band_lkr</x:v>
       </x:c>
-      <x:c r="J1" s="10" t="str">
+      <x:c r="K1" s="10" t="str">
         <x:v>rating</x:v>
       </x:c>
-      <x:c r="K1" s="10" t="str">
+      <x:c r="L1" s="10" t="str">
         <x:v>review_count</x:v>
       </x:c>
-      <x:c r="L1" s="10" t="str">
+      <x:c r="M1" s="10" t="str">
         <x:v>opening_hours</x:v>
       </x:c>
-      <x:c r="M1" s="10" t="str">
+      <x:c r="N1" s="10" t="str">
         <x:v>phone</x:v>
       </x:c>
-      <x:c r="N1" s="10" t="str">
+      <x:c r="O1" s="10" t="str">
         <x:v>signature_or_recommended_dishes</x:v>
       </x:c>
-      <x:c r="O1" s="10" t="str">
+      <x:c r="P1" s="10" t="str">
         <x:v>best_for</x:v>
       </x:c>
-      <x:c r="P1" s="10" t="str">
+      <x:c r="Q1" s="10" t="str">
         <x:v>source_type</x:v>
       </x:c>
-      <x:c r="Q1" s="10" t="str">
+      <x:c r="R1" s="10" t="str">
         <x:v>source_url</x:v>
       </x:c>
-      <x:c r="R1" s="10" t="str">
+      <x:c r="S1" s="10" t="str">
         <x:v>verified_date</x:v>
       </x:c>
-      <x:c r="S1" s="10" t="str">
+      <x:c r="T1" s="18" t="str">
         <x:v>confidence</x:v>
       </x:c>
     </x:row>
@@ -1636,51 +1656,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D2" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E2" s="11" t="str">
+      <x:c r="F2" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F2" s="11" t="str">
+      <x:c r="G2" s="11" t="str">
         <x:v>Indian / Seafood / Sri Lankan</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="H2" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H2" s="11" t="str">
+      <x:c r="I2" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I2" s="11" t="str">
+      <x:c r="J2" s="11" t="str">
         <x:v>Rs 2,000–6,000</x:v>
       </x:c>
-      <x:c r="J2" s="11" t="n">
+      <x:c r="K2" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K2" s="11" t="n">
+      <x:c r="L2" s="11" t="n">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="L2" s="11" t="str">
+      <x:c r="M2" s="11" t="str">
         <x:v>Current listing; verify day-of</x:v>
       </x:c>
-      <x:c r="M2" s="11" t="str">
+      <x:c r="N2" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N2" s="11" t="str">
+      <x:c r="O2" s="11" t="str">
         <x:v>Fresh grilled fish; seafood; authentic curries</x:v>
       </x:c>
-      <x:c r="O2" s="11" t="str">
+      <x:c r="P2" s="11" t="str">
         <x:v>fresh-catch,seafood,local-flavours</x:v>
       </x:c>
-      <x:c r="P2" s="11" t="str">
+      <x:c r="Q2" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q2" s="11" t="str">
+      <x:c r="R2" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d15073393-Reviews-The_Sketch-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R2" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S2" s="11" t="n">
+      <x:c r="S2" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T2" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>
@@ -1695,51 +1718,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D3" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E3" s="11" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F3" s="11" t="str">
+      <x:c r="G3" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="G3" s="11" t="str">
+      <x:c r="H3" s="11" t="str">
         <x:v>Medium-High</x:v>
       </x:c>
-      <x:c r="H3" s="11" t="str">
+      <x:c r="I3" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I3" s="11" t="str">
+      <x:c r="J3" s="11" t="str">
         <x:v>Rs 2,000–6,000</x:v>
       </x:c>
-      <x:c r="J3" s="11" t="n">
+      <x:c r="K3" s="11" t="n">
         <x:v>4.7</x:v>
       </x:c>
-      <x:c r="K3" s="11" t="n">
+      <x:c r="L3" s="11" t="n">
         <x:v>459</x:v>
       </x:c>
-      <x:c r="L3" s="11" t="str">
+      <x:c r="M3" s="11" t="str">
         <x:v>Current listing; verify day-of</x:v>
       </x:c>
-      <x:c r="M3" s="11" t="str">
+      <x:c r="N3" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N3" s="11" t="str">
+      <x:c r="O3" s="11" t="str">
         <x:v>Fresh fish; seafood</x:v>
       </x:c>
-      <x:c r="O3" s="11" t="str">
+      <x:c r="P3" s="11" t="str">
         <x:v>beach-seating,seafood,groups</x:v>
       </x:c>
-      <x:c r="P3" s="11" t="str">
+      <x:c r="Q3" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q3" s="11" t="str">
+      <x:c r="R3" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d12640957-Reviews-LEAF_VINE-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R3" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S3" s="11" t="n">
+      <x:c r="S3" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T3" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
     </x:row>
@@ -1754,51 +1780,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E4" s="11" t="str">
+      <x:c r="F4" s="11" t="str">
         <x:v>Cafe / seafood restaurant</x:v>
       </x:c>
-      <x:c r="F4" s="11" t="str">
+      <x:c r="G4" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="G4" s="11" t="str">
+      <x:c r="H4" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H4" s="11" t="str">
+      <x:c r="I4" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I4" s="11" t="str">
+      <x:c r="J4" s="11" t="str">
         <x:v>Budget</x:v>
       </x:c>
-      <x:c r="J4" s="11" t="n">
+      <x:c r="K4" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K4" s="11" t="n">
+      <x:c r="L4" s="11" t="n">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="L4" s="11" t="str">
+      <x:c r="M4" s="11" t="str">
         <x:v>Current listing; verify day-of</x:v>
       </x:c>
-      <x:c r="M4" s="11" t="str">
+      <x:c r="N4" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N4" s="11" t="str">
+      <x:c r="O4" s="11" t="str">
         <x:v>Prawns; calamari; white snapper</x:v>
       </x:c>
-      <x:c r="O4" s="11" t="str">
+      <x:c r="P4" s="11" t="str">
         <x:v>fresh-seafood,budget</x:v>
       </x:c>
-      <x:c r="P4" s="11" t="str">
+      <x:c r="Q4" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q4" s="11" t="str">
+      <x:c r="R4" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d20975135-Reviews-Neptune_s_Best_Restaurant_Arugambay-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R4" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S4" s="11" t="n">
+      <x:c r="S4" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T4" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>
@@ -1813,51 +1842,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E5" s="11" t="str">
+      <x:c r="F5" s="11" t="str">
         <x:v>Seafood restaurant</x:v>
       </x:c>
-      <x:c r="F5" s="11" t="str">
+      <x:c r="G5" s="11" t="str">
         <x:v>Fresh seafood / Sri Lankan</x:v>
       </x:c>
-      <x:c r="G5" s="11" t="str">
+      <x:c r="H5" s="11" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="H5" s="11" t="str">
+      <x:c r="I5" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I5" s="11" t="str">
+      <x:c r="J5" s="11" t="str">
         <x:v>Budget</x:v>
       </x:c>
-      <x:c r="J5" s="11" t="n">
+      <x:c r="K5" s="11" t="n">
         <x:v>4.6</x:v>
       </x:c>
-      <x:c r="K5" s="11" t="n">
+      <x:c r="L5" s="11" t="n">
         <x:v>1113</x:v>
       </x:c>
-      <x:c r="L5" s="11" t="str">
+      <x:c r="M5" s="11" t="str">
         <x:v>Current listing; verify day-of</x:v>
       </x:c>
-      <x:c r="M5" s="11" t="str">
+      <x:c r="N5" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N5" s="11" t="str">
+      <x:c r="O5" s="11" t="str">
         <x:v>Whole fish; prawn curry; crab; lobster</x:v>
       </x:c>
-      <x:c r="O5" s="11" t="str">
+      <x:c r="P5" s="11" t="str">
         <x:v>authentic-local,fresh-catch,seafood</x:v>
       </x:c>
-      <x:c r="P5" s="11" t="str">
+      <x:c r="Q5" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q5" s="11" t="str">
+      <x:c r="R5" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d10520610-Reviews-Mr_Fisherman-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R5" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S5" s="11" t="n">
+      <x:c r="S5" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T5" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>
@@ -1869,54 +1901,57 @@
         <x:v>Bambini's Cafe &amp; Restaurant</x:v>
       </x:c>
       <x:c r="C6" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
         <x:v>Panama Road</x:v>
       </x:c>
-      <x:c r="D6" s="11" t="str">
+      <x:c r="E6" s="11" t="str">
         <x:v>RRVJ+R74, Panama Rd, Arugam Bay</x:v>
       </x:c>
-      <x:c r="E6" s="11" t="str">
+      <x:c r="F6" s="11" t="str">
         <x:v>Cafe / restaurant</x:v>
       </x:c>
-      <x:c r="F6" s="11" t="str">
+      <x:c r="G6" s="11" t="str">
         <x:v>Seafood + mixed</x:v>
       </x:c>
-      <x:c r="G6" s="11" t="str">
+      <x:c r="H6" s="11" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="H6" s="11" t="str">
+      <x:c r="I6" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I6" s="11" t="str">
+      <x:c r="J6" s="11" t="str">
         <x:v>Rs 1,000–5,000</x:v>
       </x:c>
-      <x:c r="J6" s="11" t="n">
+      <x:c r="K6" s="11" t="n">
         <x:v>4.7</x:v>
       </x:c>
-      <x:c r="K6" s="11" t="n">
+      <x:c r="L6" s="11" t="n">
         <x:v>744</x:v>
       </x:c>
-      <x:c r="L6" s="11" t="str">
+      <x:c r="M6" s="11" t="str">
         <x:v>Open 24 hours</x:v>
       </x:c>
-      <x:c r="M6" s="11" t="str">
+      <x:c r="N6" s="11" t="str">
         <x:v>+94 77 522 6038</x:v>
       </x:c>
-      <x:c r="N6" s="11" t="str">
+      <x:c r="O6" s="11" t="str">
         <x:v>Seafood; mixed cafe meals</x:v>
       </x:c>
-      <x:c r="O6" s="11" t="str">
+      <x:c r="P6" s="11" t="str">
         <x:v>late-night,social,mixed-group</x:v>
       </x:c>
-      <x:c r="P6" s="11" t="str">
+      <x:c r="Q6" s="11" t="str">
         <x:v>Current business listing + Tripadvisor</x:v>
       </x:c>
-      <x:c r="Q6" s="11" t="str">
+      <x:c r="R6" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d10487557-Reviews-Bambini_s_Cafe-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R6" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S6" s="11" t="n">
+      <x:c r="S6" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T6" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
     </x:row>
@@ -1928,50 +1963,53 @@
         <x:v>The Green Room</x:v>
       </x:c>
       <x:c r="C7" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
         <x:v>Main Road</x:v>
       </x:c>
-      <x:c r="D7" s="11" t="str">
+      <x:c r="E7" s="11" t="str">
         <x:v>Main Road, Arugam Bay</x:v>
       </x:c>
-      <x:c r="E7" s="11" t="str">
+      <x:c r="F7" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F7" s="11" t="str">
+      <x:c r="G7" s="11" t="str">
         <x:v>Seafood / Asian / Sri Lankan</x:v>
       </x:c>
-      <x:c r="G7" s="11" t="str">
+      <x:c r="H7" s="11" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="H7" s="11" t="str">
+      <x:c r="I7" s="11" t="str">
         <x:v>Vegetarian; vegan; gluten-free listing signals</x:v>
       </x:c>
-      <x:c r="I7" s="11" t="str">
+      <x:c r="J7" s="11" t="str">
         <x:v>Budget-Mid</x:v>
       </x:c>
-      <x:c r="J7" s="11"/>
       <x:c r="K7" s="11"/>
-      <x:c r="L7" s="11" t="str">
+      <x:c r="L7" s="11"/>
+      <x:c r="M7" s="11" t="str">
         <x:v>Current page shows morning opening; verify</x:v>
       </x:c>
-      <x:c r="M7" s="11" t="str">
+      <x:c r="N7" s="11" t="str">
         <x:v>+94 77 362 6766</x:v>
       </x:c>
-      <x:c r="N7" s="11" t="str">
+      <x:c r="O7" s="11" t="str">
         <x:v>Prawn curry; garlic prawns; fish curry; fresh fish; avocado juice</x:v>
       </x:c>
-      <x:c r="O7" s="11" t="str">
+      <x:c r="P7" s="11" t="str">
         <x:v>authentic-local,seafood,dietary-inclusive</x:v>
       </x:c>
-      <x:c r="P7" s="11" t="str">
+      <x:c r="Q7" s="11" t="str">
         <x:v>Tripadvisor detailed listing</x:v>
       </x:c>
-      <x:c r="Q7" s="11" t="str">
+      <x:c r="R7" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d1733566-Reviews-The_Green_Room-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R7" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S7" s="11" t="n">
+      <x:c r="S7" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T7" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>
@@ -1983,54 +2021,57 @@
         <x:v>Curry Leaves Arugam Bay</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D8" s="11" t="str">
         <x:v>Panama Road</x:v>
       </x:c>
-      <x:c r="D8" s="11" t="str">
+      <x:c r="E8" s="11" t="str">
         <x:v>Panama Rd, Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E8" s="11" t="str">
+      <x:c r="F8" s="11" t="str">
         <x:v>Health food / Sri Lankan</x:v>
       </x:c>
-      <x:c r="F8" s="11" t="str">
+      <x:c r="G8" s="11"/>
+      <x:c r="H8" s="11" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="G8" s="11" t="str">
+      <x:c r="I8" s="11" t="str">
         <x:v>Vegetarian/health-focused</x:v>
       </x:c>
-      <x:c r="H8" s="11" t="str">
+      <x:c r="J8" s="11" t="str">
         <x:v>Mid</x:v>
       </x:c>
-      <x:c r="I8" s="11" t="n">
+      <x:c r="K8" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="J8" s="11" t="n">
+      <x:c r="L8" s="11" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="K8" s="11" t="str">
+      <x:c r="M8" s="11" t="str">
         <x:v>11:00-23:00</x:v>
       </x:c>
-      <x:c r="L8" s="11" t="str">
+      <x:c r="N8" s="11" t="str">
         <x:v>+94 76 009 6764</x:v>
       </x:c>
-      <x:c r="M8" s="11" t="str">
+      <x:c r="O8" s="11" t="str">
         <x:v>Traditional Sri Lankan food; mango curry</x:v>
       </x:c>
-      <x:c r="N8" s="11" t="str">
+      <x:c r="P8" s="11" t="str">
         <x:v>healthy,vegetarian,local-food</x:v>
       </x:c>
-      <x:c r="O8" s="11" t="str">
+      <x:c r="Q8" s="11" t="str">
         <x:v>Current business listing + Tripadvisor</x:v>
       </x:c>
-      <x:c r="P8" s="11" t="str">
+      <x:c r="R8" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d17439700-Reviews-Curry_Leaves-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="Q8" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="R8" s="11" t="n">
+      <x:c r="S8" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T8" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
-      <x:c r="S8" s="11"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="11" t="str">
@@ -2040,54 +2081,57 @@
         <x:v>Dosa Station</x:v>
       </x:c>
       <x:c r="C9" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D9" s="11" t="str">
         <x:v>Main Street</x:v>
       </x:c>
-      <x:c r="D9" s="11" t="str">
+      <x:c r="E9" s="11" t="str">
         <x:v>Main Street, Arugam Bay 32506</x:v>
       </x:c>
-      <x:c r="E9" s="11" t="str">
+      <x:c r="F9" s="11" t="str">
         <x:v>Sri Lankan / South Indian restaurant</x:v>
       </x:c>
-      <x:c r="F9" s="11" t="str">
+      <x:c r="G9" s="11" t="str">
         <x:v>Tamil / South Indian / Sri Lankan</x:v>
       </x:c>
-      <x:c r="G9" s="11" t="str">
+      <x:c r="H9" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H9" s="11" t="str">
+      <x:c r="I9" s="11" t="str">
         <x:v>Strong vegetarian potential</x:v>
       </x:c>
-      <x:c r="I9" s="11" t="str">
+      <x:c r="J9" s="11" t="str">
         <x:v>Rs 1,000–2,000</x:v>
       </x:c>
-      <x:c r="J9" s="11" t="n">
+      <x:c r="K9" s="11" t="n">
         <x:v>4.8</x:v>
       </x:c>
-      <x:c r="K9" s="11" t="n">
+      <x:c r="L9" s="11" t="n">
         <x:v>1036</x:v>
       </x:c>
-      <x:c r="L9" s="11" t="str">
+      <x:c r="M9" s="11" t="str">
         <x:v>08:00-23:00; Fri split hours</x:v>
       </x:c>
-      <x:c r="M9" s="11" t="str">
+      <x:c r="N9" s="11" t="str">
         <x:v>+94 75 819 3653</x:v>
       </x:c>
-      <x:c r="N9" s="11" t="str">
+      <x:c r="O9" s="11" t="str">
         <x:v>Dosa; vegetarian meals</x:v>
       </x:c>
-      <x:c r="O9" s="11" t="str">
+      <x:c r="P9" s="11" t="str">
         <x:v>vegetarian,budget,tamil-food</x:v>
       </x:c>
-      <x:c r="P9" s="11" t="str">
+      <x:c r="Q9" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q9" s="11" t="str">
+      <x:c r="R9" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Dosa+Station+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R9" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S9" s="11" t="n">
+      <x:c r="S9" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T9" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
     </x:row>
@@ -2099,54 +2143,57 @@
         <x:v>Dewa Restaurant &amp; Cafe</x:v>
       </x:c>
       <x:c r="C10" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D10" s="11" t="str">
         <x:v>Panama Road</x:v>
       </x:c>
-      <x:c r="D10" s="11" t="str">
+      <x:c r="E10" s="11" t="str">
         <x:v>RRVJ+R74, Panama Rd, Arugam Bay</x:v>
       </x:c>
-      <x:c r="E10" s="11" t="str">
+      <x:c r="F10" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F10" s="11" t="str">
+      <x:c r="G10" s="11" t="str">
         <x:v>Seafood / beach dining</x:v>
       </x:c>
-      <x:c r="G10" s="11" t="str">
+      <x:c r="H10" s="11" t="str">
         <x:v>Medium-High</x:v>
       </x:c>
-      <x:c r="H10" s="11" t="str">
+      <x:c r="I10" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I10" s="11" t="str">
+      <x:c r="J10" s="11" t="str">
         <x:v>Rs 2,000–7,000</x:v>
       </x:c>
-      <x:c r="J10" s="11" t="n">
+      <x:c r="K10" s="11" t="n">
         <x:v>4.7</x:v>
       </x:c>
-      <x:c r="K10" s="11" t="n">
+      <x:c r="L10" s="11" t="n">
         <x:v>2014</x:v>
       </x:c>
-      <x:c r="L10" s="11" t="str">
+      <x:c r="M10" s="11" t="str">
         <x:v>07:30-23:00</x:v>
       </x:c>
-      <x:c r="M10" s="11" t="str">
+      <x:c r="N10" s="11" t="str">
         <x:v>+94 71 949 4360</x:v>
       </x:c>
-      <x:c r="N10" s="11" t="str">
+      <x:c r="O10" s="11" t="str">
         <x:v>Fresh seafood platters; cocktails</x:v>
       </x:c>
-      <x:c r="O10" s="11" t="str">
+      <x:c r="P10" s="11" t="str">
         <x:v>seafood,beach-dining,groups</x:v>
       </x:c>
-      <x:c r="P10" s="11" t="str">
+      <x:c r="Q10" s="11" t="str">
         <x:v>Official website + current business listing</x:v>
       </x:c>
-      <x:c r="Q10" s="11" t="str">
+      <x:c r="R10" s="11" t="str">
         <x:v>https://dewasrilanka.com/</x:v>
       </x:c>
-      <x:c r="R10" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S10" s="11" t="n">
+      <x:c r="S10" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T10" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>
@@ -2158,54 +2205,57 @@
         <x:v>CATCH OF THE DAY</x:v>
       </x:c>
       <x:c r="C11" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D11" s="11" t="str">
         <x:v>Panama Road</x:v>
       </x:c>
-      <x:c r="D11" s="11" t="str">
+      <x:c r="E11" s="11" t="str">
         <x:v>Panama Rd, Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E11" s="11" t="str">
+      <x:c r="F11" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F11" s="11" t="str">
+      <x:c r="G11" s="11" t="str">
         <x:v>Seafood / fresh catch</x:v>
       </x:c>
-      <x:c r="G11" s="11" t="str">
+      <x:c r="H11" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H11" s="11" t="str">
+      <x:c r="I11" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I11" s="11" t="str">
+      <x:c r="J11" s="11" t="str">
         <x:v>Rs 3,000–4,000</x:v>
       </x:c>
-      <x:c r="J11" s="11" t="n">
+      <x:c r="K11" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K11" s="11" t="n">
+      <x:c r="L11" s="11" t="n">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="L11" s="11" t="str">
+      <x:c r="M11" s="11" t="str">
         <x:v>11:00-23:00</x:v>
       </x:c>
-      <x:c r="M11" s="11" t="str">
+      <x:c r="N11" s="11" t="str">
         <x:v>+94 74 373 7997</x:v>
       </x:c>
-      <x:c r="N11" s="11" t="str">
+      <x:c r="O11" s="11" t="str">
         <x:v>Fresh catch seafood</x:v>
       </x:c>
-      <x:c r="O11" s="11" t="str">
+      <x:c r="P11" s="11" t="str">
         <x:v>fresh-catch,seafood</x:v>
       </x:c>
-      <x:c r="P11" s="11" t="str">
+      <x:c r="Q11" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q11" s="11" t="str">
+      <x:c r="R11" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Catch+of+the+Day+Arugam+Bay+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R11" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S11" s="11" t="n">
+      <x:c r="S11" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T11" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
     </x:row>
@@ -2217,54 +2267,57 @@
         <x:v>Haliaeetus Seafood Restaurant Arugambay</x:v>
       </x:c>
       <x:c r="C12" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D12" s="11" t="str">
         <x:v>Pottuvil / Arugam Bay area</x:v>
       </x:c>
-      <x:c r="D12" s="11" t="str">
+      <x:c r="E12" s="11" t="str">
         <x:v>Arugam Bay area</x:v>
       </x:c>
-      <x:c r="E12" s="11" t="str">
+      <x:c r="F12" s="11" t="str">
         <x:v>Seafood restaurant</x:v>
       </x:c>
-      <x:c r="F12" s="11" t="str">
+      <x:c r="G12" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="G12" s="11" t="str">
+      <x:c r="H12" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H12" s="11" t="str">
+      <x:c r="I12" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I12" s="11" t="str">
+      <x:c r="J12" s="11" t="str">
         <x:v>Budget-Mid</x:v>
       </x:c>
-      <x:c r="J12" s="11" t="n">
+      <x:c r="K12" s="11" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K12" s="11" t="n">
+      <x:c r="L12" s="11" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="L12" s="11" t="str">
+      <x:c r="M12" s="11" t="str">
         <x:v>Current listing; verify</x:v>
       </x:c>
-      <x:c r="M12" s="11" t="str">
+      <x:c r="N12" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N12" s="11" t="str">
+      <x:c r="O12" s="11" t="str">
         <x:v>Fresh fish and seafood</x:v>
       </x:c>
-      <x:c r="O12" s="11" t="str">
+      <x:c r="P12" s="11" t="str">
         <x:v>fresh-catch,seafood,quiet</x:v>
       </x:c>
-      <x:c r="P12" s="11" t="str">
+      <x:c r="Q12" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q12" s="11" t="str">
+      <x:c r="R12" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d33095308-Reviews-Haliaeetus_Seafood_Restaurant_Arugambay-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R12" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S12" s="11" t="n">
+      <x:c r="S12" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T12" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2279,51 +2332,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E13" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E13" s="11" t="str">
+      <x:c r="F13" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F13" s="11" t="str">
+      <x:c r="G13" s="11" t="str">
         <x:v>Seafood / mixed</x:v>
       </x:c>
-      <x:c r="G13" s="11" t="str">
+      <x:c r="H13" s="11" t="str">
         <x:v>Medium-High</x:v>
       </x:c>
-      <x:c r="H13" s="11" t="str">
+      <x:c r="I13" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I13" s="11" t="str">
+      <x:c r="J13" s="11" t="str">
         <x:v>Rs 2,000–6,000</x:v>
       </x:c>
-      <x:c r="J13" s="11" t="n">
+      <x:c r="K13" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K13" s="11" t="n">
+      <x:c r="L13" s="11" t="n">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="L13" s="11" t="str">
+      <x:c r="M13" s="11" t="str">
         <x:v>Current listing; verify</x:v>
       </x:c>
-      <x:c r="M13" s="11" t="str">
+      <x:c r="N13" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N13" s="11" t="str">
+      <x:c r="O13" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="O13" s="11" t="str">
+      <x:c r="P13" s="11" t="str">
         <x:v>seafood,modern,groups</x:v>
       </x:c>
-      <x:c r="P13" s="11" t="str">
+      <x:c r="Q13" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q13" s="11" t="str">
+      <x:c r="R13" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d33036335-Reviews-Wave_Arugam_Bay-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R13" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S13" s="11" t="n">
+      <x:c r="S13" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T13" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2338,51 +2394,54 @@
         <x:v>Arugam Bay</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="E14" s="11" t="str">
         <x:v>Arugam Bay, Eastern Province</x:v>
       </x:c>
-      <x:c r="E14" s="11" t="str">
+      <x:c r="F14" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F14" s="11" t="str">
+      <x:c r="G14" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="G14" s="11" t="str">
+      <x:c r="H14" s="11" t="str">
         <x:v>Medium-High</x:v>
       </x:c>
-      <x:c r="H14" s="11" t="str">
+      <x:c r="I14" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I14" s="11" t="str">
+      <x:c r="J14" s="11" t="str">
         <x:v>Rs 2,000–6,000</x:v>
       </x:c>
-      <x:c r="J14" s="11" t="n">
+      <x:c r="K14" s="11" t="n">
         <x:v>4.6</x:v>
       </x:c>
-      <x:c r="K14" s="11" t="n">
+      <x:c r="L14" s="11" t="n">
         <x:v>179</x:v>
       </x:c>
-      <x:c r="L14" s="11" t="str">
+      <x:c r="M14" s="11" t="str">
         <x:v>Current listing; verify</x:v>
       </x:c>
-      <x:c r="M14" s="11" t="str">
+      <x:c r="N14" s="11" t="str">
         <x:v>Not reliably listed</x:v>
       </x:c>
-      <x:c r="N14" s="11" t="str">
+      <x:c r="O14" s="11" t="str">
         <x:v>Seafood platter; prawns; calamari</x:v>
       </x:c>
-      <x:c r="O14" s="11" t="str">
+      <x:c r="P14" s="11" t="str">
         <x:v>beach-dining,seafood</x:v>
       </x:c>
-      <x:c r="P14" s="11" t="str">
+      <x:c r="Q14" s="11" t="str">
         <x:v>Tripadvisor current listing</x:v>
       </x:c>
-      <x:c r="Q14" s="11" t="str">
+      <x:c r="R14" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d23910391-Reviews-Serendib_Arugam_Bay-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R14" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S14" s="11" t="n">
+      <x:c r="S14" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T14" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2394,54 +2453,57 @@
         <x:v>Shady Lane</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D15" s="11" t="str">
         <x:v>Sinhapura Road</x:v>
       </x:c>
-      <x:c r="D15" s="11" t="str">
+      <x:c r="E15" s="11" t="str">
         <x:v>RRPP+786, Sinhapura Rd, Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E15" s="11" t="str">
+      <x:c r="F15" s="11" t="str">
         <x:v>Cafe</x:v>
       </x:c>
-      <x:c r="F15" s="11" t="str">
+      <x:c r="G15" s="11" t="str">
         <x:v>Vegetarian / cafe</x:v>
       </x:c>
-      <x:c r="G15" s="11" t="str">
+      <x:c r="H15" s="11" t="str">
         <x:v>Low local-food strength</x:v>
       </x:c>
-      <x:c r="H15" s="11" t="str">
+      <x:c r="I15" s="11" t="str">
         <x:v>Vegetarian / vegan-friendly cafe profile</x:v>
       </x:c>
-      <x:c r="I15" s="11" t="str">
+      <x:c r="J15" s="11" t="str">
         <x:v>Mid</x:v>
       </x:c>
-      <x:c r="J15" s="11" t="n">
+      <x:c r="K15" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K15" s="11" t="n">
+      <x:c r="L15" s="11" t="n">
         <x:v>525</x:v>
       </x:c>
-      <x:c r="L15" s="11" t="str">
+      <x:c r="M15" s="11" t="str">
         <x:v>Verify current branch hours</x:v>
       </x:c>
-      <x:c r="M15" s="11" t="str">
+      <x:c r="N15" s="11" t="str">
         <x:v>+94 77 082 5420</x:v>
       </x:c>
-      <x:c r="N15" s="11" t="str">
+      <x:c r="O15" s="11" t="str">
         <x:v>Breakfast; cafe dishes; smoothies</x:v>
       </x:c>
-      <x:c r="O15" s="11" t="str">
+      <x:c r="P15" s="11" t="str">
         <x:v>vegetarian,breakfast,surf-cafe</x:v>
       </x:c>
-      <x:c r="P15" s="11" t="str">
+      <x:c r="Q15" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q15" s="11" t="str">
+      <x:c r="R15" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Shady+Lane+Arugam+Bay+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R15" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S15" s="11" t="n">
+      <x:c r="S15" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T15" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2453,54 +2515,57 @@
         <x:v>Curry Leaves Arugam Bay</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D16" s="11" t="str">
         <x:v>Panama Road</x:v>
       </x:c>
-      <x:c r="D16" s="11" t="str">
+      <x:c r="E16" s="11" t="str">
         <x:v>Panama Rd, Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E16" s="11" t="str">
+      <x:c r="F16" s="11" t="str">
         <x:v>Health food restaurant</x:v>
       </x:c>
-      <x:c r="F16" s="11" t="str">
+      <x:c r="G16" s="11" t="str">
         <x:v>Sri Lankan / healthy</x:v>
       </x:c>
-      <x:c r="G16" s="11" t="str">
+      <x:c r="H16" s="11" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="H16" s="11" t="str">
+      <x:c r="I16" s="11" t="str">
         <x:v>Vegetarian-friendly</x:v>
       </x:c>
-      <x:c r="I16" s="11" t="str">
+      <x:c r="J16" s="11" t="str">
         <x:v>Rs 2,000–3,000</x:v>
       </x:c>
-      <x:c r="J16" s="11" t="n">
+      <x:c r="K16" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K16" s="11" t="n">
+      <x:c r="L16" s="11" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="L16" s="11" t="str">
+      <x:c r="M16" s="11" t="str">
         <x:v>11:00-23:00</x:v>
       </x:c>
-      <x:c r="M16" s="11" t="str">
+      <x:c r="N16" s="11" t="str">
         <x:v>+94 76 009 6764</x:v>
       </x:c>
-      <x:c r="N16" s="11" t="str">
+      <x:c r="O16" s="11" t="str">
         <x:v>Mango curry; traditional Sri Lankan dishes</x:v>
       </x:c>
-      <x:c r="O16" s="11" t="str">
+      <x:c r="P16" s="11" t="str">
         <x:v>healthy,local-food,vegetarian</x:v>
       </x:c>
-      <x:c r="P16" s="11" t="str">
+      <x:c r="Q16" s="11" t="str">
         <x:v>Current business + Tripadvisor</x:v>
       </x:c>
-      <x:c r="Q16" s="11" t="str">
+      <x:c r="R16" s="11" t="str">
         <x:v>https://www.tripadvisor.com/Restaurant_Review-g3348959-d17439700-Reviews-Curry_Leaves-Arugam_Bay_Eastern_Province.html</x:v>
       </x:c>
-      <x:c r="R16" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S16" s="11" t="n">
+      <x:c r="S16" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T16" s="11" t="n">
         <x:v>0.98</x:v>
       </x:c>
     </x:row>
@@ -2512,54 +2577,57 @@
         <x:v>Surf Resort Beach Restaurant</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="str">
         <x:v>Beach area</x:v>
       </x:c>
-      <x:c r="D17" s="11" t="str">
+      <x:c r="E17" s="11" t="str">
         <x:v>Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E17" s="11" t="str">
+      <x:c r="F17" s="11" t="str">
         <x:v>Seafood restaurant</x:v>
       </x:c>
-      <x:c r="F17" s="11" t="str">
+      <x:c r="G17" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="G17" s="11" t="str">
+      <x:c r="H17" s="11" t="str">
         <x:v>Medium-High</x:v>
       </x:c>
-      <x:c r="H17" s="11" t="str">
+      <x:c r="I17" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I17" s="11" t="str">
+      <x:c r="J17" s="11" t="str">
         <x:v>Rs 2,000–6,000</x:v>
       </x:c>
-      <x:c r="J17" s="11" t="n">
+      <x:c r="K17" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K17" s="11" t="n">
+      <x:c r="L17" s="11" t="n">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="L17" s="11" t="str">
+      <x:c r="M17" s="11" t="str">
         <x:v>07:00-23:30</x:v>
       </x:c>
-      <x:c r="M17" s="11" t="str">
+      <x:c r="N17" s="11" t="str">
         <x:v>+94 77 780 4272</x:v>
       </x:c>
-      <x:c r="N17" s="11" t="str">
+      <x:c r="O17" s="11" t="str">
         <x:v>Seafood</x:v>
       </x:c>
-      <x:c r="O17" s="11" t="str">
+      <x:c r="P17" s="11" t="str">
         <x:v>beach-dining,seafood</x:v>
       </x:c>
-      <x:c r="P17" s="11" t="str">
+      <x:c r="Q17" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q17" s="11" t="str">
+      <x:c r="R17" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Surf+Resort+Beach+Restaurant+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R17" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S17" s="11" t="n">
+      <x:c r="S17" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T17" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2571,54 +2639,57 @@
         <x:v>Fish Corner Restaurant</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="str">
         <x:v>Main Street</x:v>
       </x:c>
-      <x:c r="D18" s="11" t="str">
+      <x:c r="E18" s="11" t="str">
         <x:v>Main Street, Arugam Bay</x:v>
       </x:c>
-      <x:c r="E18" s="11" t="str">
+      <x:c r="F18" s="11" t="str">
         <x:v>Restaurant</x:v>
       </x:c>
-      <x:c r="F18" s="11" t="str">
+      <x:c r="G18" s="11" t="str">
         <x:v>Seafood / local</x:v>
       </x:c>
-      <x:c r="G18" s="11" t="str">
+      <x:c r="H18" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H18" s="11" t="str">
+      <x:c r="I18" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I18" s="11" t="str">
+      <x:c r="J18" s="11" t="str">
         <x:v>Rs 3,000–4,000</x:v>
       </x:c>
-      <x:c r="J18" s="11" t="n">
+      <x:c r="K18" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K18" s="11" t="n">
+      <x:c r="L18" s="11" t="n">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="L18" s="11" t="str">
+      <x:c r="M18" s="11" t="str">
         <x:v>24 hours</x:v>
       </x:c>
-      <x:c r="M18" s="11" t="str">
+      <x:c r="N18" s="11" t="str">
         <x:v>+94 75 271 5665</x:v>
       </x:c>
-      <x:c r="N18" s="11" t="str">
+      <x:c r="O18" s="11" t="str">
         <x:v>Fresh fish; seafood</x:v>
       </x:c>
-      <x:c r="O18" s="11" t="str">
+      <x:c r="P18" s="11" t="str">
         <x:v>late-night,seafood,fresh-catch</x:v>
       </x:c>
-      <x:c r="P18" s="11" t="str">
+      <x:c r="Q18" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q18" s="11" t="str">
+      <x:c r="R18" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Fish+Corner+Restaurant+Arugam+Bay+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R18" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S18" s="11" t="n">
+      <x:c r="S18" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T18" s="11" t="n">
         <x:v>0.96</x:v>
       </x:c>
     </x:row>
@@ -2630,54 +2701,57 @@
         <x:v>Banana Surf Cafe</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D19" s="11" t="str">
         <x:v>Main Street</x:v>
       </x:c>
-      <x:c r="D19" s="11" t="str">
+      <x:c r="E19" s="11" t="str">
         <x:v>Main Street, Arugam Bay 32500</x:v>
       </x:c>
-      <x:c r="E19" s="11" t="str">
+      <x:c r="F19" s="11" t="str">
         <x:v>Cafe</x:v>
       </x:c>
-      <x:c r="F19" s="11" t="str">
+      <x:c r="G19" s="11" t="str">
         <x:v>Cafe / breakfast</x:v>
       </x:c>
-      <x:c r="G19" s="11" t="str">
+      <x:c r="H19" s="11" t="str">
         <x:v>Low local-food strength</x:v>
       </x:c>
-      <x:c r="H19" s="11" t="str">
+      <x:c r="I19" s="11" t="str">
         <x:v>Mixed</x:v>
       </x:c>
-      <x:c r="I19" s="11" t="str">
+      <x:c r="J19" s="11" t="str">
         <x:v>Rs 2,000–3,000</x:v>
       </x:c>
-      <x:c r="J19" s="11" t="n">
+      <x:c r="K19" s="11" t="n">
         <x:v>4.9</x:v>
       </x:c>
-      <x:c r="K19" s="11" t="n">
+      <x:c r="L19" s="11" t="n">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="L19" s="11" t="str">
+      <x:c r="M19" s="11" t="str">
         <x:v>07:30-17:00</x:v>
       </x:c>
-      <x:c r="M19" s="11" t="str">
+      <x:c r="N19" s="11" t="str">
         <x:v>+94 77 540 7670</x:v>
       </x:c>
-      <x:c r="N19" s="11" t="str">
+      <x:c r="O19" s="11" t="str">
         <x:v>Breakfast; cafe food</x:v>
       </x:c>
-      <x:c r="O19" s="11" t="str">
+      <x:c r="P19" s="11" t="str">
         <x:v>breakfast,surf-cafe</x:v>
       </x:c>
-      <x:c r="P19" s="11" t="str">
+      <x:c r="Q19" s="11" t="str">
         <x:v>Current business listing</x:v>
       </x:c>
-      <x:c r="Q19" s="11" t="str">
+      <x:c r="R19" s="11" t="str">
         <x:v>https://www.google.com/maps/search/?api=1&amp;query=Banana+Surf+Cafe+Arugam+Bay+Arugam+Bay+Sri+Lanka</x:v>
       </x:c>
-      <x:c r="R19" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S19" s="11" t="n">
+      <x:c r="S19" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T19" s="11" t="n">
         <x:v>0.95</x:v>
       </x:c>
     </x:row>
@@ -2689,50 +2763,53 @@
         <x:v>Beach Hut Dinner</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D20" s="11" t="str">
         <x:v>Arugam Bay beach area</x:v>
       </x:c>
-      <x:c r="D20" s="11" t="str">
+      <x:c r="E20" s="11" t="str">
         <x:v>Arugam Bay</x:v>
       </x:c>
-      <x:c r="E20" s="11" t="str">
+      <x:c r="F20" s="11" t="str">
         <x:v>Guesthouse dinner / communal meal</x:v>
       </x:c>
-      <x:c r="F20" s="11" t="str">
+      <x:c r="G20" s="11" t="str">
         <x:v>Sri Lankan / BBQ</x:v>
       </x:c>
-      <x:c r="G20" s="11" t="str">
+      <x:c r="H20" s="11" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="H20" s="11" t="str">
+      <x:c r="I20" s="11" t="str">
         <x:v>Menu varies</x:v>
       </x:c>
-      <x:c r="I20" s="11" t="str">
+      <x:c r="J20" s="11" t="str">
         <x:v>Budget</x:v>
       </x:c>
-      <x:c r="J20" s="11"/>
       <x:c r="K20" s="11"/>
-      <x:c r="L20" s="11" t="str">
+      <x:c r="L20" s="11"/>
+      <x:c r="M20" s="11" t="str">
         <x:v>Evening set-menu; verify current schedule</x:v>
       </x:c>
-      <x:c r="M20" s="11" t="str">
+      <x:c r="N20" s="11" t="str">
         <x:v>Not listed</x:v>
       </x:c>
-      <x:c r="N20" s="11" t="str">
+      <x:c r="O20" s="11" t="str">
         <x:v>Fish BBQ; changing set dinner</x:v>
       </x:c>
-      <x:c r="O20" s="11" t="str">
+      <x:c r="P20" s="11" t="str">
         <x:v>social,bbq,budget,backpacker</x:v>
       </x:c>
-      <x:c r="P20" s="11" t="str">
+      <x:c r="Q20" s="11" t="str">
         <x:v>Travel guide</x:v>
       </x:c>
-      <x:c r="Q20" s="11" t="str">
+      <x:c r="R20" s="11" t="str">
         <x:v>https://www.thecoastalcampaign.com/arugam-bay-things-to-do/</x:v>
       </x:c>
-      <x:c r="R20" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S20" s="11" t="n">
+      <x:c r="S20" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T20" s="11" t="n">
         <x:v>0.84</x:v>
       </x:c>
     </x:row>
@@ -2744,50 +2821,53 @@
         <x:v>Cook with Mona</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
+        <x:v>Arugam Bay</x:v>
+      </x:c>
+      <x:c r="D21" s="11" t="str">
         <x:v>Arugam Bay village</x:v>
       </x:c>
-      <x:c r="D21" s="11" t="str">
+      <x:c r="E21" s="11" t="str">
         <x:v>Traditional home setting in Arugam Bay</x:v>
       </x:c>
-      <x:c r="E21" s="11" t="str">
+      <x:c r="F21" s="11" t="str">
         <x:v>Cooking class / home dining</x:v>
       </x:c>
-      <x:c r="F21" s="11" t="str">
+      <x:c r="G21" s="11" t="str">
         <x:v>Sri Lankan</x:v>
       </x:c>
-      <x:c r="G21" s="11" t="str">
+      <x:c r="H21" s="11" t="str">
         <x:v>Very High</x:v>
       </x:c>
-      <x:c r="H21" s="11" t="str">
+      <x:c r="I21" s="11" t="str">
         <x:v>Can adapt dishes; verify dietary needs</x:v>
       </x:c>
-      <x:c r="I21" s="11" t="str">
+      <x:c r="J21" s="11" t="str">
         <x:v>Experience-based</x:v>
       </x:c>
-      <x:c r="J21" s="11"/>
       <x:c r="K21" s="11"/>
-      <x:c r="L21" s="11" t="str">
+      <x:c r="L21" s="11"/>
+      <x:c r="M21" s="11" t="str">
         <x:v>Class/session based</x:v>
       </x:c>
-      <x:c r="M21" s="11" t="str">
+      <x:c r="N21" s="11" t="str">
         <x:v>Not listed</x:v>
       </x:c>
-      <x:c r="N21" s="11" t="str">
+      <x:c r="O21" s="11" t="str">
         <x:v>Rice and curry; coconut roti; coconut sambol; bean/pumpkin/chicken curry</x:v>
       </x:c>
-      <x:c r="O21" s="11" t="str">
+      <x:c r="P21" s="11" t="str">
         <x:v>cooking-class,authentic-local,cultural-experience</x:v>
       </x:c>
-      <x:c r="P21" s="11" t="str">
+      <x:c r="Q21" s="11" t="str">
         <x:v>Official website + Instagram</x:v>
       </x:c>
-      <x:c r="Q21" s="11" t="str">
+      <x:c r="R21" s="11" t="str">
         <x:v>https://cookwithmonaarugambay.wordpress.com/</x:v>
       </x:c>
-      <x:c r="R21" s="11" t="str">
-        <x:v>2026-08-11</x:v>
-      </x:c>
-      <x:c r="S21" s="11" t="n">
+      <x:c r="S21" s="11" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="T21" s="11" t="n">
         <x:v>0.99</x:v>
       </x:c>
     </x:row>

</xml_diff>